<commit_message>
Test update tinh.xlsx data
</commit_message>
<xml_diff>
--- a/tinh.xlsx
+++ b/tinh.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VKSNDTC\Projects\thongkenhaplieu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VisualCodeWorkspace\PythonWeb\thongkenhaplieu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD33C7C-4475-42D9-B629-4D281B5DF22B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEFB753-D837-4DE7-BF74-D104846B343E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8BD0CAC4-3BA0-4DC6-9391-9CBA79D907C0}"/>
+    <workbookView xWindow="27636" yWindow="1488" windowWidth="17280" windowHeight="8880" xr2:uid="{8BD0CAC4-3BA0-4DC6-9391-9CBA79D907C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -638,6 +638,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33BBBD07-AF56-4FFB-A2BF-B2E8A6A9EBD7}">
   <dimension ref="A1:M36"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="51" thickBot="1">
       <c r="A1" s="1" t="s">
@@ -1716,7 +1719,7 @@
         <v>13</v>
       </c>
       <c r="D27" s="9">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="E27" s="10">
         <v>1.0210148641722194</v>

</xml_diff>